<commit_message>
ПМИ dtz1 и dtz2
</commit_message>
<xml_diff>
--- a/PMI-DZT2/ПМИ ДЗТ/pmi_dzt/dtz1_mode/ДТЗ_6.xlsx
+++ b/PMI-DZT2/ПМИ ДЗТ/pmi_dzt/dtz1_mode/ДТЗ_6.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -46,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,21 +51,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -465,135 +453,135 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>TDIF_1_Side1</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>TDIF_1_Side2</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>TDIF_1_Side3</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>TDIF_1_KschemeSide1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>TDIF_1_KschemeSide2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>TDIF_1_KschemeSide3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>TDIF_1_Equaliz3I0s1</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>TDIF_1_Equaliz3I0s2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TDIF_1_Equaliz3I0s3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_EnaDis</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_EnaDis_ctbreak</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_EnaDis</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_EnaDis_ctbreak</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_EnaDis</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_EnaDis_ctbreak</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_EnaDis</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_RstMod</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_EnaDisSelec</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_EnaDis</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_RegBlock</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_RegBlock</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_EnaDis</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_PTRC1_EnaDis</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_RBRE1_EnaDis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
@@ -632,10 +620,10 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="Q2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="R2" t="n">
@@ -653,10 +641,10 @@
       <c r="V2" t="n">
         <v>0</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="X2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -728,257 +716,257 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_Tbrk</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_Tasym</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_Inom</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_Imin</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_Ksym</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_LIsym</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_Tbrk</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_Tasym</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_Inom</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_Imin</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_Ksym</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_LIsym</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_Tbrk</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_Tasym</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_Inom</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_Imin</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_Ksym</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_LIsym</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>TDIF_1_Sbase</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>TDIF_1_Unom1</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>TDIF_1_Unom2</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>TDIF_1_Unom3</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>TDIF_1_IprimSide1</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>TDIF_1_IprimSide2</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>TDIF_1_IprimSide3</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>TDIF_1_Inomterm1</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>TDIF_1_Inomterm2</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>TDIF_1_Inomterm3</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>TDIF_1_IsecSide1</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>TDIF_1_IsecSide2</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>TDIF_1_IsecSide3</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>TDIF_1_ConnGr1</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>TDIF_1_ConnGr2</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>TDIF_1_ConnGr3</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Top</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Iop</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_IopCSS</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Irest1</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Irest2</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Krest1</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Krest2</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_Top</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_Iop</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Tret</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Tblock</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_K2Hdiv1H</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Tret</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Tblock</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_K5Hdiv1H</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_Top</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_Iop</t>
         </is>
@@ -991,16 +979,16 @@
       <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="1" t="n">
         <v>0.05</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>0.02</v>
       </c>
       <c r="G2" t="n">
@@ -1009,16 +997,16 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>0.05</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" s="1" t="n">
         <v>0.02</v>
       </c>
       <c r="M2" t="n">
@@ -1027,115 +1015,115 @@
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="O2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="1" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="Q2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="R2" s="2" t="n">
+      <c r="R2" s="1" t="n">
         <v>0.02</v>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="S2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="T2" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="U2" s="1" t="n">
         <v>10.5</v>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="V2" s="1" t="n">
         <v>10.5</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" s="1" t="n">
         <v>750</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="X2" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="Y2" s="2" t="n">
+      <c r="Y2" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="Z2" s="2" t="n">
+      <c r="Z2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AA2" s="2" t="n">
+      <c r="AA2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AB2" s="2" t="n">
+      <c r="AB2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AC2" s="2" t="n">
+      <c r="AC2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AD2" s="2" t="n">
+      <c r="AD2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="AE2" s="2" t="n">
+      <c r="AE2" s="1" t="n">
         <v>5</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
       </c>
-      <c r="AG2" s="2" t="n">
+      <c r="AG2" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="AH2" s="2" t="n">
+      <c r="AH2" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="AI2" s="2" t="n">
+      <c r="AI2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AJ2" s="2" t="n">
+      <c r="AJ2" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="AK2" s="2" t="n">
+      <c r="AK2" s="1" t="n">
         <v>1.2</v>
       </c>
-      <c r="AL2" s="2" t="n">
+      <c r="AL2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AM2" s="2" t="n">
+      <c r="AM2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="AN2" s="2" t="n">
+      <c r="AN2" s="1" t="n">
         <v>0.25</v>
       </c>
-      <c r="AO2" s="2" t="n">
+      <c r="AO2" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="AP2" s="2" t="n">
+      <c r="AP2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AQ2" s="2" t="n">
+      <c r="AQ2" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="AR2" s="2" t="n">
+      <c r="AR2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AS2" s="2" t="n">
+      <c r="AS2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AT2" s="2" t="n">
+      <c r="AT2" s="1" t="n">
         <v>0.2</v>
       </c>
-      <c r="AU2" s="2" t="n">
+      <c r="AU2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AV2" s="2" t="n">
+      <c r="AV2" s="1" t="n">
         <v>0.5</v>
       </c>
-      <c r="AW2" s="2" t="n">
+      <c r="AW2" s="1" t="n">
         <v>0.3</v>
       </c>
-      <c r="AX2" s="2" t="n">
+      <c r="AX2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="AY2" s="2" t="n">
+      <c r="AY2" s="1" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1188,162 +1176,162 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>DI_ControllerDisable</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>DI_CTR_UIRZ</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>DI_CTR_RCTR1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>DI_CTR_RCTR2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DI_CTR_RCTR3</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DI_TDIF</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DI_RESPDIF</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>DI_RESPDIF_Sign</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>DI_INSPDIF</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>DI_INSPDIF_Sign</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>DI_ATDIFRCTR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>DI_TPRMOFFLVLGC</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>DI_TJNTPTRC</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>DI_JNTRBRE</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dIA</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>IB</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dIB</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>dIC</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>IA1</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>dIA1</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>IB1</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>dIB1</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>IC1</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>dIC1</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>IA2harm</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>IB2harm</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>IC2harm</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>IA5harm</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>IB5harm</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>IC5harm</t>
         </is>
@@ -1371,7 +1359,7 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="n">
@@ -1392,22 +1380,22 @@
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="O2" s="1" t="n">
         <v>1.1</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="Q2" s="1" t="n">
         <v>1.1</v>
       </c>
-      <c r="R2" s="2" t="n">
+      <c r="R2" s="1" t="n">
         <v>240</v>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="S2" s="1" t="n">
         <v>1.1</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="T2" s="1" t="n">
         <v>120</v>
       </c>
       <c r="U2" t="n">
@@ -1419,13 +1407,13 @@
       <c r="W2" t="n">
         <v>0</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="X2" s="1" t="n">
         <v>240</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" s="2" t="n">
+      <c r="Z2" s="1" t="n">
         <v>120</v>
       </c>
       <c r="AA2" t="n">
@@ -1546,412 +1534,412 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_FuncEnabled</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_StrBrkCF</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_OpBrkCF</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_StrAsymCF</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR1_OpAsymCF</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_FuncEnabled</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_StrBrkCF</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_OpBrkCF</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_StrAsymCF</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR2_OpAsymCF</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_FuncEnabled</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_StrBrkCF</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_OpBrkCF</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_StrAsymCF</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_RCTR3_OpAsymCF</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>CTR_UIRZ_1_CTR_UIRZ_CurCircFlt</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_FuncEnabled</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_StrPhA</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhA</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhAOnSignal</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_DE_IA</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_StrPhB</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhB</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhBOnSignal</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_DE_IB</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_StrPhC</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhC</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpPhCOnSignal</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_DE_IC</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_Str</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_OpOnSignal</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF2_Op</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_FuncEnabled</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_StrPhA</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhA</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhAOnSignal</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_DE_IA</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_StrPhB</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhB</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhBOnSignal</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_DE_IB</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_StrPhC</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhC</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpPhCOnSignal</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_DE_IC</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Str</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_OpOnSignal</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>TDIF_1_PDIF1_Op</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Str2HIa</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Str2HIb</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Str2HIc</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>TDIF_1_HF2PHAR1_Str2H</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Str5HIa</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Str5HIb</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Str5HIc</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>TDIF_1_HF5PHAR1_Str5H</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_FuncEnabled</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_CurCircAlmPhA</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_CurCircAlmPhB</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_CurCircAlmPhC</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_CurCircAlm</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>TDIF_1_RCTR1_CurCircFltGen</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_PTRC1_FuncEnabled</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_PTRC1_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>pusk_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_PTRC1_Op</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_RBRE1_FuncEnabled</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_RBRE1_FuncOperDisabled</t>
         </is>
       </c>
-      <c r="BW1" s="1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>TPRMOFFLVLGC_1_RBRE1_BlkOp</t>
         </is>
       </c>
-      <c r="BX1" s="1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>DZT2_LVALH_1_CALH1_Alarm</t>
         </is>
       </c>
-      <c r="BY1" s="1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>diffA</t>
         </is>
       </c>
-      <c r="BZ1" s="1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>restA</t>
         </is>
       </c>
-      <c r="CA1" s="1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>diffB</t>
         </is>
       </c>
-      <c r="CB1" s="1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>restB</t>
         </is>
       </c>
-      <c r="CC1" s="1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>diffC</t>
         </is>
       </c>
-      <c r="CD1" s="1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>restC</t>
         </is>
@@ -2138,7 +2126,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AK2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2148,7 +2136,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
+      <c r="AM2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2158,17 +2146,17 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AO2" s="2" t="inlineStr">
+      <c r="AO2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AP2" s="2" t="inlineStr">
+      <c r="AP2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AQ2" s="2" t="inlineStr">
+      <c r="AQ2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2178,17 +2166,17 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AS2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AT2" s="2" t="inlineStr">
+      <c r="AT2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AU2" s="2" t="inlineStr">
+      <c r="AU2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2198,22 +2186,22 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AW2" s="2" t="inlineStr">
+      <c r="AW2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AX2" s="2" t="inlineStr">
+      <c r="AX2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AY2" s="2" t="inlineStr">
+      <c r="AY2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AZ2" s="2" t="inlineStr">
+      <c r="AZ2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2298,7 +2286,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="BQ2" s="2" t="inlineStr">
+      <c r="BQ2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2318,7 +2306,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="BU2" s="2" t="inlineStr">
+      <c r="BU2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2333,39 +2321,39 @@
           <t>0</t>
         </is>
       </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BY2" s="2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="BZ2" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="CA2" s="2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="CB2" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="CC2" s="2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="CD2" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
+      <c r="BX2" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BY2" s="1" t="inlineStr">
+        <is>
+          <t>1000.26</t>
+        </is>
+      </c>
+      <c r="BZ2" s="1" t="inlineStr">
+        <is>
+          <t>500.13</t>
+        </is>
+      </c>
+      <c r="CA2" s="1" t="inlineStr">
+        <is>
+          <t>1000.26</t>
+        </is>
+      </c>
+      <c r="CB2" s="1" t="inlineStr">
+        <is>
+          <t>500.13</t>
+        </is>
+      </c>
+      <c r="CC2" s="1" t="inlineStr">
+        <is>
+          <t>1000.26</t>
+        </is>
+      </c>
+      <c r="CD2" s="1" t="inlineStr">
+        <is>
+          <t>500.13</t>
         </is>
       </c>
     </row>

</xml_diff>